<commit_message>
Track AFL Solar Sox clients (Diaz, Tookoian, Dominick Reid).
Resolve Dominick Reid via Stats API id, label Arizona Fall League assignments, and point schedules at the dated AFL scores hub.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/client_lists/Client List - 04-15-26.xlsx
+++ b/client_lists/Client List - 04-15-26.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
-  <dimension ref="A1:G120"/>
+  <dimension ref="A1:H120"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="24.6640625" customWidth="1" style="4" min="1" max="1"/>
@@ -2446,7 +2446,7 @@
     <row r="66">
       <c r="A66" s="3" t="inlineStr">
         <is>
-          <t>Reid, Dom</t>
+          <t>Reid, Dominick</t>
         </is>
       </c>
       <c r="B66" s="3" t="inlineStr">

</xml_diff>